<commit_message>
Smartphone survey data for PCA
</commit_message>
<xml_diff>
--- a/data/Processed/Participant_details.xlsx
+++ b/data/Processed/Participant_details.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28129"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28429"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\ecf-exp2-notif-mmn\data\Processed\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{418E47D9-1405-456B-B802-892A58895DD6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{27EA0A75-C75B-4553-A416-88BC7AB2CE45}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="33120" yWindow="1305" windowWidth="21600" windowHeight="11385" xr2:uid="{96E66801-AEE8-4A11-9971-0DA162AB42F9}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{96E66801-AEE8-4A11-9971-0DA162AB42F9}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="204" uniqueCount="57">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="240" uniqueCount="65">
   <si>
     <t>SN</t>
   </si>
@@ -210,6 +210,30 @@
   </si>
   <si>
     <t>non_acd</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> </t>
+  </si>
+  <si>
+    <t>SD041</t>
+  </si>
+  <si>
+    <t>SD042</t>
+  </si>
+  <si>
+    <t>SD043</t>
+  </si>
+  <si>
+    <t>SD044</t>
+  </si>
+  <si>
+    <t>SD045</t>
+  </si>
+  <si>
+    <t>SD046</t>
+  </si>
+  <si>
+    <t>SD047</t>
   </si>
 </sst>
 </file>
@@ -590,7 +614,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{865CEB74-C7CC-4BC7-8922-8A1352A31C27}">
-  <dimension ref="A1:I40"/>
+  <dimension ref="A1:L47"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="6.42578125" style="1" customWidth="1"/>
@@ -1533,7 +1557,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="33" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A33" s="1">
         <v>32</v>
       </c>
@@ -1541,7 +1565,7 @@
         <v>36</v>
       </c>
       <c r="C33" s="1">
-        <v>27</v>
+        <v>36</v>
       </c>
       <c r="D33" s="1" t="s">
         <v>45</v>
@@ -1561,8 +1585,11 @@
       <c r="I33" s="1" t="s">
         <v>56</v>
       </c>
-    </row>
-    <row r="34" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="L33" s="1" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="34" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A34" s="1">
         <v>33</v>
       </c>
@@ -1570,7 +1597,7 @@
         <v>37</v>
       </c>
       <c r="C34" s="1">
-        <v>36</v>
+        <v>27</v>
       </c>
       <c r="D34" s="1" t="s">
         <v>45</v>
@@ -1591,7 +1618,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="35" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A35" s="1">
         <v>34</v>
       </c>
@@ -1620,7 +1647,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="36" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A36" s="1">
         <v>35</v>
       </c>
@@ -1649,7 +1676,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="37" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A37" s="1">
         <v>36</v>
       </c>
@@ -1678,7 +1705,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="38" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A38" s="1">
         <v>37</v>
       </c>
@@ -1707,7 +1734,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="39" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A39" s="1">
         <v>38</v>
       </c>
@@ -1736,7 +1763,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="40" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A40" s="1">
         <v>39</v>
       </c>
@@ -1763,6 +1790,209 @@
       </c>
       <c r="I40" s="1" t="s">
         <v>56</v>
+      </c>
+    </row>
+    <row r="41" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A41" s="1">
+        <v>40</v>
+      </c>
+      <c r="B41" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="C41" s="1">
+        <v>34</v>
+      </c>
+      <c r="D41" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="E41" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="F41" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="G41" s="1">
+        <v>156</v>
+      </c>
+      <c r="H41" s="1">
+        <v>143</v>
+      </c>
+      <c r="I41" s="1" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="42" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A42" s="1">
+        <v>41</v>
+      </c>
+      <c r="B42" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="C42" s="1">
+        <v>38</v>
+      </c>
+      <c r="D42" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="E42" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="F42" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="G42" s="1">
+        <v>156</v>
+      </c>
+      <c r="H42" s="1">
+        <v>140</v>
+      </c>
+      <c r="I42" s="1" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="43" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A43" s="1">
+        <v>42</v>
+      </c>
+      <c r="B43" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="C43" s="1">
+        <v>28</v>
+      </c>
+      <c r="D43" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="E43" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="F43" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="G43" s="1">
+        <v>110</v>
+      </c>
+      <c r="H43" s="1">
+        <v>103</v>
+      </c>
+      <c r="I43" s="1" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="44" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A44" s="1">
+        <v>43</v>
+      </c>
+      <c r="B44" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="C44" s="1">
+        <v>26</v>
+      </c>
+      <c r="D44" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="E44" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="F44" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="G44" s="1">
+        <v>124</v>
+      </c>
+      <c r="H44" s="1">
+        <v>91</v>
+      </c>
+      <c r="I44" s="1" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="45" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A45" s="1">
+        <v>44</v>
+      </c>
+      <c r="B45" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="C45" s="1">
+        <v>26</v>
+      </c>
+      <c r="D45" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="E45" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="F45" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="G45" s="1">
+        <v>152</v>
+      </c>
+      <c r="H45" s="1">
+        <v>101</v>
+      </c>
+      <c r="I45" s="1" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="46" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A46" s="1">
+        <v>45</v>
+      </c>
+      <c r="B46" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="C46" s="1">
+        <v>23</v>
+      </c>
+      <c r="D46" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="E46" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="F46" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="G46" s="1">
+        <v>102</v>
+      </c>
+      <c r="H46" s="1">
+        <v>76</v>
+      </c>
+      <c r="I46" s="1" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="47" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A47" s="1">
+        <v>46</v>
+      </c>
+      <c r="B47" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="C47" s="1">
+        <v>26</v>
+      </c>
+      <c r="D47" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="E47" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="F47" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="G47" s="1">
+        <v>128</v>
+      </c>
+      <c r="H47" s="1">
+        <v>105</v>
+      </c>
+      <c r="I47" s="1" t="s">
+        <v>54</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Block 2 issuse for the delayed triggers
</commit_message>
<xml_diff>
--- a/data/Processed/Participant_details.xlsx
+++ b/data/Processed/Participant_details.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29029"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\ecf-exp2-notif-mmn\data\Processed\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7664F962-A936-48AB-889F-EFC601272E57}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{16B16392-DE4E-46D2-9DCE-69E40F0CDF0A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{96E66801-AEE8-4A11-9971-0DA162AB42F9}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="488" uniqueCount="123">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="488" uniqueCount="124">
   <si>
     <t>gender</t>
   </si>
@@ -368,9 +368,6 @@
     <t>bad electrode =PO4</t>
   </si>
   <si>
-    <t>bad electrode =AF7, PO7, PO3</t>
-  </si>
-  <si>
     <t>bad electrode = PO7</t>
   </si>
   <si>
@@ -386,9 +383,6 @@
     <t>bad electrode = P5</t>
   </si>
   <si>
-    <t xml:space="preserve">Droped </t>
-  </si>
-  <si>
     <t xml:space="preserve">bad electrode = FC3; it have additional S24 ,S25 trgger reponse </t>
   </si>
   <si>
@@ -408,6 +402,15 @@
   </si>
   <si>
     <t>bad electrode = CP5, Fp2, C1</t>
+  </si>
+  <si>
+    <t>bad electrode = ['AF7', 'PO4', 'PO3', 'FT9', 'F2']</t>
+  </si>
+  <si>
+    <t>bad electrode =['AF7', 'Fp1', 'F6', 'AF8', 'FC3', 'PO3', 'TP7', 'P5', 'PO7']</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> ['PO3', 'P6', 'F4', 'Oz', 'FT9'] Dropped </t>
   </si>
 </sst>
 </file>
@@ -1802,13 +1805,13 @@
         <v>79</v>
       </c>
       <c r="G32" s="1" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="H32" s="1" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I32" s="2" t="s">
-        <v>77</v>
+        <v>121</v>
       </c>
       <c r="J32" s="1" t="s">
         <v>84</v>
@@ -1980,7 +1983,7 @@
         <v>6</v>
       </c>
       <c r="I37" s="2" t="s">
-        <v>109</v>
+        <v>122</v>
       </c>
       <c r="J37" s="1" t="s">
         <v>98</v>
@@ -2015,7 +2018,7 @@
         <v>6</v>
       </c>
       <c r="I38" s="2" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="J38" s="1" t="s">
         <v>98</v>
@@ -2050,7 +2053,7 @@
         <v>6</v>
       </c>
       <c r="I39" s="2" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="J39" s="1" t="s">
         <v>99</v>
@@ -2111,10 +2114,10 @@
         <v>3</v>
       </c>
       <c r="F41" s="1" t="s">
-        <v>79</v>
+        <v>7</v>
       </c>
       <c r="G41" s="1" t="s">
-        <v>7</v>
+        <v>79</v>
       </c>
       <c r="H41" s="1" t="s">
         <v>6</v>
@@ -2190,7 +2193,7 @@
         <v>6</v>
       </c>
       <c r="I43" s="2" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="J43" s="1" t="s">
         <v>85</v>
@@ -2295,7 +2298,7 @@
         <v>6</v>
       </c>
       <c r="I46" s="2" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="J46" s="1" t="s">
         <v>82</v>
@@ -2400,7 +2403,7 @@
         <v>6</v>
       </c>
       <c r="I49" s="2" t="s">
-        <v>115</v>
+        <v>123</v>
       </c>
       <c r="J49" s="1" t="s">
         <v>95</v>
@@ -2435,7 +2438,7 @@
         <v>6</v>
       </c>
       <c r="I50" s="2" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="J50" s="1" t="s">
         <v>91</v>
@@ -2505,7 +2508,7 @@
         <v>6</v>
       </c>
       <c r="I52" s="2" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="J52" s="1" t="s">
         <v>99</v>
@@ -2540,7 +2543,7 @@
         <v>6</v>
       </c>
       <c r="I53" s="2" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="J53" s="1" t="s">
         <v>92</v>
@@ -2575,7 +2578,7 @@
         <v>6</v>
       </c>
       <c r="I54" s="2" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="J54" s="1" t="s">
         <v>98</v>
@@ -2610,7 +2613,7 @@
         <v>6</v>
       </c>
       <c r="I55" s="2" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="J55" s="1" t="s">
         <v>99</v>
@@ -2680,7 +2683,7 @@
         <v>6</v>
       </c>
       <c r="I57" s="2" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="J57" s="1" t="s">
         <v>97</v>
@@ -2715,7 +2718,7 @@
         <v>6</v>
       </c>
       <c r="I58" s="2" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="J58" s="1" t="s">
         <v>81</v>
@@ -2726,7 +2729,7 @@
     </row>
     <row r="60" spans="1:15" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="O60" s="1" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
     </row>
     <row r="63" spans="1:15" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Rearrange the notebooks and SME analysis
</commit_message>
<xml_diff>
--- a/data/Processed/Participant_details.xlsx
+++ b/data/Processed/Participant_details.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\ecf-exp2-notif-mmn\data\Processed\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{16B16392-DE4E-46D2-9DCE-69E40F0CDF0A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AFC46F4F-6BF6-4479-9E8A-272CE7B6B779}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{96E66801-AEE8-4A11-9971-0DA162AB42F9}"/>
+    <workbookView xWindow="31170" yWindow="0" windowWidth="29040" windowHeight="15840" xr2:uid="{96E66801-AEE8-4A11-9971-0DA162AB42F9}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="488" uniqueCount="124">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="488" uniqueCount="125">
   <si>
     <t>gender</t>
   </si>
@@ -383,9 +383,6 @@
     <t>bad electrode = P5</t>
   </si>
   <si>
-    <t xml:space="preserve">bad electrode = FC3; it have additional S24 ,S25 trgger reponse </t>
-  </si>
-  <si>
     <t>bad electrode = FT7</t>
   </si>
   <si>
@@ -404,20 +401,86 @@
     <t>bad electrode = CP5, Fp2, C1</t>
   </si>
   <si>
-    <t>bad electrode = ['AF7', 'PO4', 'PO3', 'FT9', 'F2']</t>
-  </si>
-  <si>
-    <t>bad electrode =['AF7', 'Fp1', 'F6', 'AF8', 'FC3', 'PO3', 'TP7', 'P5', 'PO7']</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> ['PO3', 'P6', 'F4', 'Oz', 'FT9'] Dropped </t>
+    <t>bad electrode = FC3; it have additional S24 ,S25 trgger reponse ; further don't have psycho data to shift as system stopped before saving the results</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">bad electrode =['AF7', 'Fp1', 'F6', 'AF8', 'FC3', 'PO3', 'TP7', 'P5', 'PO7'];  The EEG trigger for the Control block is 21, 22, 23, 24, and 25, whereas for PS as the standard tone has stimulus markers with 31, 32, 33, 34, and 35. </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Corrected</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>bad electrode = ['AF7', 'PO4', 'PO3', 'FT9', 'F2'] ; Control Block EEG is collected at  the end with trigger value similar to personlized tone as EEG recoring was not resumed in actual place.</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> Corrected</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">bad electrode = None; Each block of data is collected by interchanging the tone in first block so need not to shift movie to sound trigger.  </t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve"> ['P5', 'P6','F5',  'Oz', 'FT9'] </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Dropped ; lot of noise</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> ;The recording system closed after two blocks. The third block (beep tone as deviant ) is recorded in a separate file SD058_B3.eeg. </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">Raw data corrected </t>
+    </r>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -431,13 +494,33 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.39997558519241921"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -452,12 +535,18 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1810,8 +1899,8 @@
       <c r="H32" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I32" s="2" t="s">
-        <v>121</v>
+      <c r="I32" s="3" t="s">
+        <v>122</v>
       </c>
       <c r="J32" s="1" t="s">
         <v>84</v>
@@ -1982,8 +2071,8 @@
       <c r="H37" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="I37" s="2" t="s">
-        <v>122</v>
+      <c r="I37" s="3" t="s">
+        <v>121</v>
       </c>
       <c r="J37" s="1" t="s">
         <v>98</v>
@@ -2367,8 +2456,8 @@
       <c r="H48" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="I48" s="2" t="s">
-        <v>77</v>
+      <c r="I48" s="3" t="s">
+        <v>123</v>
       </c>
       <c r="J48" s="1" t="s">
         <v>94</v>
@@ -2402,8 +2491,8 @@
       <c r="H49" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="I49" s="2" t="s">
-        <v>123</v>
+      <c r="I49" s="3" t="s">
+        <v>124</v>
       </c>
       <c r="J49" s="1" t="s">
         <v>95</v>
@@ -2479,7 +2568,7 @@
         <v>96</v>
       </c>
       <c r="K51" s="1">
-        <v>2.9251700680272101E-3</v>
+        <v>2.9251699999999999E-3</v>
       </c>
     </row>
     <row r="52" spans="1:15" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
@@ -2507,8 +2596,8 @@
       <c r="H52" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="I52" s="2" t="s">
-        <v>114</v>
+      <c r="I52" s="4" t="s">
+        <v>120</v>
       </c>
       <c r="J52" s="1" t="s">
         <v>99</v>
@@ -2543,7 +2632,7 @@
         <v>6</v>
       </c>
       <c r="I53" s="2" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="J53" s="1" t="s">
         <v>92</v>
@@ -2578,7 +2667,7 @@
         <v>6</v>
       </c>
       <c r="I54" s="2" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="J54" s="1" t="s">
         <v>98</v>
@@ -2613,7 +2702,7 @@
         <v>6</v>
       </c>
       <c r="I55" s="2" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="J55" s="1" t="s">
         <v>99</v>
@@ -2683,7 +2772,7 @@
         <v>6</v>
       </c>
       <c r="I57" s="2" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="J57" s="1" t="s">
         <v>97</v>
@@ -2718,7 +2807,7 @@
         <v>6</v>
       </c>
       <c r="I58" s="2" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="J58" s="1" t="s">
         <v>81</v>
@@ -2729,7 +2818,7 @@
     </row>
     <row r="60" spans="1:15" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="O60" s="1" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
     </row>
     <row r="63" spans="1:15" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">

</xml_diff>